<commit_message>
Docker setup for deployment
</commit_message>
<xml_diff>
--- a/llm_stats/token_usage.xlsx
+++ b/llm_stats/token_usage.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX7"/>
+  <dimension ref="A1:AX10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1960,6 +1960,692 @@
       </c>
       <c r="AX7" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>d30a2a88-986d-40ef-a051-cc94482a3ed2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-03-12 21:30:04</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>3622</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Check Divisibility by Digit Sum and Product</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/check-divisibility-by-digit-sum-and-product/description/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>mistral</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>analysis_only_append_code_v1</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>190d07deeba31923371931835131a7c933cda0cea82e762a7fb575ee0620409f</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>You are an expert technical writer creating a high-quality LeetCode solution post. Problem Details: Number: 3622 Name: Check Divisibility by Digit Sum and Product Difficulty: easy Link: https://leetcode.com/problems/check-divisibility-by-digit-sum-and-product/description/ Pyth...</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are an expert technical writer creating a high-quality LeetCode solution post.
+Problem Details:
+Number: 3622
+Name: Check Divisibility by Digit Sum and Product
+Difficulty: easy
+Link: https://leetcode.com/problems/check-divisibility-by-digit-sum-and-product/description/
+Python Solution:
+class Solution:
+    def checkDivisibility(self, n: int) -&gt; bool:
+        presDigitSum = 0
+        presDigitProduct = 1
+        originalNo = n
+        while n &gt; 0:
+            presDigit = n%10
+            presDigitSum += presDigit
+            presDigitProduct *= presDigit
+            n = n//10
+        return originalNo%(presDigitSum+presDigitProduct) == 0
+Instructions:
+1. Generate a strong, descriptive, professional Title.
+- The title MUST mention:
+    - The core technique used
+    - The time complexity (Big-O notation)
+- The explanation must match the provided language
+- IMPORTANT: The title text (after "Title: ") must be 75 characters or fewer.
+2. Generate markdown using exactly these sections and no additional top-level sections:
+Title: &lt;single line title, max 75 characters&gt;
+## Intuition
+## Approach
+## Time Complexity
+## Space Complexity
+3. Do NOT include any code block and do NOT add a ## Code section.
+4. Keep the response concise, technical, and ready for markdown publishing.
+</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1302</v>
+      </c>
+      <c r="O8" t="n">
+        <v>42</v>
+      </c>
+      <c r="P8" t="n">
+        <v>366</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>13</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>be052ed46c2d8207e2a263b065073525ffce218711af2c625d5b3e6f4316532b</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>class Solution:
+    def checkDivisibility(self, n: int) -&gt; bool:
+        presDigitSum = 0
+        presDigitProduct = 1
+        originalNo = n
+        while n &gt; 0:
+            presDigit = n%10
+            presDigitSum += presDigit
+            presDigitProduct *= presDigit
+            n = n//10
+        return originalNo%(presDigitSum+presDigitProduct) == 0</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>379</v>
+      </c>
+      <c r="U8" t="n">
+        <v>327</v>
+      </c>
+      <c r="V8" t="n">
+        <v>706</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.8628</v>
+      </c>
+      <c r="X8" t="n">
+        <v>97439.44</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>8465.74</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>30790.23</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>57369.32</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>5.6999</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>1372</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>22</v>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>Title: Divisibility Check Using Digit Sum and Product in Python (O(log n))
+## Intuition
+The problem requires checking if a number `n` is divisible by the sum of its digits plus the product of its digits. The algorithm iteratively calculates both quantities as we traverse the number, comparing them to the original number at each step to determine divisibility.
+## Approach
+1. Initialize variables for storing the partial digit sum and product during traversal of the input number `n`.
+2. Iterate through each digit in the number from right to left. In each iteration:
+   - Add the current digit to the partial sum (`presDigitSum`).
+   - Multiply the partial product (`presDigitProduct`) by the current digit.
+   - Divide `n` by 10 to remove its least significant digit and use the result for the next iteration.
+3. Return True if the original number is divisible by the calculated sum and product, and False otherwise.
+## Time Complexity
+The time complexity of this solution is O(log n), since we traverse the input number logarithmically using integer division (//). The constant factor involved in this solution is relatively small due to minimal arithmetic operations per iteration.
+## Space Complexity
+The space complexity of this solution is O(1) as it uses only a few constants and variables, which do not increase based on the size of the input number `n`.</t>
+        </is>
+      </c>
+      <c r="AL8" t="n">
+        <v>1839</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>42</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>100</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>100</v>
+      </c>
+      <c r="AX8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9adeffbb-cdd7-4e54-bb87-ec6d2e3abd36</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-03-12 21:31:12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>704</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Binary Search</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/binary-search/description/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>mistral</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>analysis_only_append_code_v1</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>4c1920be931a0e0f286bac0b10ab71359af3866862bfefe062950718493bd2e4</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>You are an expert technical writer creating a high-quality LeetCode solution post. Problem Details: Number: 704 Name: Binary Search Difficulty: easy Link: https://leetcode.com/problems/binary-search/description/ Python Solution: import bisect class Solution: def search(self, n...</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are an expert technical writer creating a high-quality LeetCode solution post.
+Problem Details:
+Number: 704
+Name: Binary Search
+Difficulty: easy
+Link: https://leetcode.com/problems/binary-search/description/
+Python Solution:
+import bisect
+class Solution:
+    def search(self, nums: List[int], target: int) -&gt; int:
+        index = bisect.bisect_left(nums,target)
+        if index &lt; len(nums):
+            if nums[index] == target:
+                return index
+        return -1
+Instructions:
+1. Generate a strong, descriptive, professional Title.
+- The title MUST mention:
+    - The core technique used
+    - The time complexity (Big-O notation)
+- The explanation must match the provided language
+- IMPORTANT: The title text (after "Title: ") must be 75 characters or fewer.
+2. Generate markdown using exactly these sections and no additional top-level sections:
+Title: &lt;single line title, max 75 characters&gt;
+## Intuition
+## Approach
+## Time Complexity
+## Space Complexity
+3. Do NOT include any code block and do NOT add a ## Code section.
+4. Keep the response concise, technical, and ready for markdown publishing.
+</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1129</v>
+      </c>
+      <c r="O9" t="n">
+        <v>40</v>
+      </c>
+      <c r="P9" t="n">
+        <v>254</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>11</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>e137afb35da73117914419ecea6d521e1c376640a9bf108fd31f9c25d0bfff60</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>import bisect
+class Solution:
+    def search(self, nums: List[int], target: int) -&gt; int:
+        index = bisect.bisect_left(nums,target)
+        if index &lt; len(nums):
+            if nums[index] == target:
+                return index
+        return -1</t>
+        </is>
+      </c>
+      <c r="T9" t="n">
+        <v>324</v>
+      </c>
+      <c r="U9" t="n">
+        <v>264</v>
+      </c>
+      <c r="V9" t="n">
+        <v>588</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.8148</v>
+      </c>
+      <c r="X9" t="n">
+        <v>165410.18</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>8464.709999999999</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>23870.55</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>43291.78</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>6.0982</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>1202</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>17</v>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>Title: Binary Search Using Bisect in Python - O(log n) Time Complexity
+## Intuition
+The binary search algorithm is a divide-and-conquer method used for finding an element within a sorted list by repeatedly dividing the search interval in half. This strategy makes it an efficient solution when dealing with large datasets.
+## Approach
+In this implementation, we utilize the built-in `bisect` module in Python to perform a binary search. The `bisect_left` function finds the insertion point for target in sorted list nums such that all elements before it are less than or equal to target. If the found index has a matching value with target, it is returned; otherwise, -1 is returned.
+## Time Complexity
+The time complexity of this approach is O(log n) because each comparison eliminates half of the remaining elements in the sorted list. This makes binary search one of the most efficient searching algorithms for large datasets.
+## Space Complexity
+In terms of space complexity, our solution requires only a constant amount of additional space (O(1)) for the `index` variable since it simply keeps track of the search progress without storing all intermediate values during the search process.</t>
+        </is>
+      </c>
+      <c r="AL9" t="n">
+        <v>1557</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>35</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>100</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>100</v>
+      </c>
+      <c r="AX9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>a877842e-dc7c-4d06-b988-654259a0d3b1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-03-12 21:32:51</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2236</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Root Equals Sum of Children</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/root-equals-sum-of-children/description/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>mistral</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>analysis_only_append_code_v1</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>6f78255f768bfa5f0cae2b19b49b5e9ac4f4ccad222b54f97c0804076b85421e</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>You are an expert technical writer creating a high-quality LeetCode solution post. Problem Details: Number: 2236 Name: Root Equals Sum of Children Difficulty: easy Link: https://leetcode.com/problems/root-equals-sum-of-children/description/ Python Solution: # Definition for a ...</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are an expert technical writer creating a high-quality LeetCode solution post.
+Problem Details:
+Number: 2236
+Name: Root Equals Sum of Children
+Difficulty: easy
+Link: https://leetcode.com/problems/root-equals-sum-of-children/description/
+Python Solution:
+# Definition for a binary tree node.
+# class TreeNode:
+#     def __init__(self, val=0, left=None, right=None):
+#         self.val = val
+#         self.left = left
+#         self.right = right
+class Solution:
+    def checkTree(self, root: Optional[TreeNode]) -&gt; bool:
+        if not root:
+            return True
+        rootVal = root.val
+        leftVal, rightVal = 0,0
+        if root.left:
+            leftVal = root.left.val
+        if root.right:
+            rightVal = root.right.val
+        return rootVal == leftVal + rightVal
+Instructions:
+1. Generate a strong, descriptive, professional Title.
+- The title MUST mention:
+    - The core technique used
+    - The time complexity (Big-O notation)
+- The explanation must match the provided language
+- IMPORTANT: The title text (after "Title: ") must be 75 characters or fewer.
+2. Generate markdown using exactly these sections and no additional top-level sections:
+Title: &lt;single line title, max 75 characters&gt;
+## Intuition
+## Approach
+## Time Complexity
+## Space Complexity
+3. Do NOT include any code block and do NOT add a ## Code section.
+4. Keep the response concise, technical, and ready for markdown publishing.
+</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1450</v>
+      </c>
+      <c r="O10" t="n">
+        <v>50</v>
+      </c>
+      <c r="P10" t="n">
+        <v>546</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>21</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>788ab863539fc469928f080678dccaa087cbb6071486d394a933156490bf5d20</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t># Definition for a binary tree node.
+# class TreeNode:
+#     def __init__(self, val=0, left=None, right=None):
+#         self.val = val
+#         self.left = left
+#         self.right = right
+class Solution:
+    def checkTree(self, root: Optional[TreeNode]) -&gt; bool:
+        if not root:
+            return True
+        rootVal = root.val
+        leftVal, rightVal = 0,0
+        if root.left:
+            leftVal = root.left.val
+        if root.right:
+            rightVal = root.right.val
+        return rootVal == leftVal + rightVal</t>
+        </is>
+      </c>
+      <c r="T10" t="n">
+        <v>416</v>
+      </c>
+      <c r="U10" t="n">
+        <v>349</v>
+      </c>
+      <c r="V10" t="n">
+        <v>765</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.8389</v>
+      </c>
+      <c r="X10" t="n">
+        <v>263537.47</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>8464.709999999999</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>32888.37</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>64436.57</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>5.4162</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>1395</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>17</v>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>Title: Depth-First Search Verification: O(N) Solution for LeetCode Problem 2236
+## Intuition
+The core technique employed in this solution is a depth-first search (DFS). The goal is to verify if the root value of a binary tree equals the sum of its children's values. We perform DFS on the tree to calculate the sum of both children recursively, then compare it with the root's value.
+## Approach
+Starting from the root node, we recursively traverse the binary tree using DFS. At each level (either left or right subtree), we calculate the sum of all nodes' values. When reaching the leaf nodes, we return the calculated sum as the sum of its children. Finally, we compare this sum with the root's value and check if they are equal. If yes, the tree satisfies the condition; otherwise, it does not.
+## Time Complexity
+The time complexity of our solution is O(N), where N is the number of nodes in the binary tree. This is due to the recursive nature of DFS, which visits each node only once.
+## Space Complexity
+The space complexity of this algorithm is O(H), where H is the height of the tree. We utilize the stack to store the recursion call frames during the DFS traversal, and the maximum depth reached in the traversal will define the stack's size. However, since it's a balanced binary tree, the height is logarithmic (O(log N)), hence the overall space complexity is also O(log N).</t>
+        </is>
+      </c>
+      <c r="AL10" t="n">
+        <v>2042</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>45</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>100</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>100</v>
+      </c>
+      <c r="AX10" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1993,7 +2679,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -2003,7 +2689,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -2033,7 +2719,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5.58</v>
+        <v>5.64</v>
       </c>
     </row>
     <row r="7">
@@ -2043,7 +2729,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>122902.86</v>
+        <v>140422.7</v>
       </c>
     </row>
     <row r="8">
@@ -2053,7 +2739,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>97.22</v>
+        <v>98.15000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -2063,7 +2749,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>96.67</v>
+        <v>97.78</v>
       </c>
     </row>
   </sheetData>
@@ -2077,7 +2763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2211,7 +2897,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4136b715d00f86dbecec596bc2b3edd9d641459ca344c6cf63430eeb8a8d0479</t>
+          <t>190d07deeba31923371931835131a7c933cda0cea82e762a7fb575ee0620409f</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -2224,10 +2910,10 @@
         <v>100</v>
       </c>
       <c r="H4" t="n">
-        <v>6.08</v>
+        <v>5.7</v>
       </c>
       <c r="I4" t="n">
-        <v>1.1103</v>
+        <v>0.8628</v>
       </c>
     </row>
     <row r="5">
@@ -2248,7 +2934,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>bc4d6a1b30057aeb421828e3058b67b393c68ef3e9a044f87d681c404bd8d7c3</t>
+          <t>4136b715d00f86dbecec596bc2b3edd9d641459ca344c6cf63430eeb8a8d0479</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -2261,10 +2947,10 @@
         <v>100</v>
       </c>
       <c r="H5" t="n">
-        <v>6.31</v>
+        <v>6.08</v>
       </c>
       <c r="I5" t="n">
-        <v>0.9457</v>
+        <v>1.1103</v>
       </c>
     </row>
     <row r="6">
@@ -2285,7 +2971,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>c0cf95285f54eaebedb9669a2aebe8239832722a8830a2e4215272d5a7af2264</t>
+          <t>4c1920be931a0e0f286bac0b10ab71359af3866862bfefe062950718493bd2e4</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -2298,9 +2984,120 @@
         <v>100</v>
       </c>
       <c r="H6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.8148</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>analysis_only_append_code_v1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>mistral</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>6f78255f768bfa5f0cae2b19b49b5e9ac4f4ccad222b54f97c0804076b85421e</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.8389</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>analysis_only_append_code_v1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>mistral</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>bc4d6a1b30057aeb421828e3058b67b393c68ef3e9a044f87d681c404bd8d7c3</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>100</v>
+      </c>
+      <c r="G8" t="n">
+        <v>100</v>
+      </c>
+      <c r="H8" t="n">
+        <v>6.31</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.9457</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>v1.0.0</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>analysis_only_append_code_v1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>mistral</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>c0cf95285f54eaebedb9669a2aebe8239832722a8830a2e4215272d5a7af2264</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H9" t="n">
         <v>4.64</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I9" t="n">
         <v>1.1983</v>
       </c>
     </row>
@@ -2352,16 +3149,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
-        <v>5.58</v>
+        <v>5.64</v>
       </c>
       <c r="D2" t="n">
-        <v>122902.86</v>
+        <v>140422.7</v>
       </c>
       <c r="E2" t="n">
-        <v>97.22</v>
+        <v>98.15000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>